<commit_message>
fix: [special approval] amount validation
</commit_message>
<xml_diff>
--- a/src/assets/template/RDD-OIT-180-Template.xlsx
+++ b/src/assets/template/RDD-OIT-180-Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dxcportal.sharepoint.com/sites/philipschinaapps/SpecialApproval/1.Requirement Phase/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="287" documentId="8_{900191A1-6134-4C80-866E-A4E3C8406C5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20517C06-D02F-4267-AAE9-28B280EB49E9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1C7867-598C-463B-AA01-AC07CD155279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{A3335066-89F2-47A1-BD65-2F9EA0750B57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{A3335066-89F2-47A1-BD65-2F9EA0750B57}"/>
   </bookViews>
   <sheets>
     <sheet name="RDD&gt; 180 " sheetId="3" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RDD&gt; 180 with fields Type'!$B$2:$AP$2</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -65,153 +66,153 @@
   <commentList>
     <comment ref="F1" authorId="0" shapeId="0" xr:uid="{B4B208CB-0F9D-4DC1-8613-8805F940725B}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="G1" authorId="1" shapeId="0" xr:uid="{6F20C107-C597-4385-BDB4-D9A9983767C2}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="H1" authorId="2" shapeId="0" xr:uid="{A132152D-919D-40B2-8C2A-0E6484404566}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="I1" authorId="3" shapeId="0" xr:uid="{11083C8A-3F35-45FC-9AAC-05A74C2F7FA9}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="J1" authorId="4" shapeId="0" xr:uid="{CD547CB8-656D-457B-89E3-EB9FFFB9C968}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="M1" authorId="5" shapeId="0" xr:uid="{0FEE6189-3BC3-49AA-8D5C-86B06582D8C0}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new add</t>
       </text>
     </comment>
     <comment ref="N1" authorId="6" shapeId="0" xr:uid="{D08BAA86-3079-4ECE-8723-BF407AACEDD2}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new add</t>
       </text>
     </comment>
     <comment ref="P1" authorId="7" shapeId="0" xr:uid="{B85CD7DF-9270-48D8-995A-A030AFB0A36F}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new add</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="8" shapeId="0" xr:uid="{88B9159E-C49E-4602-A429-3800654CD8F1}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new add</t>
       </text>
     </comment>
     <comment ref="R1" authorId="9" shapeId="0" xr:uid="{745D14E2-9168-4628-89D9-5FD3462F45C4}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="S1" authorId="10" shapeId="0" xr:uid="{5906C2E1-A890-48D6-A4C0-040ED15032CD}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="T1" authorId="11" shapeId="0" xr:uid="{4A9B8EBD-80C2-4F39-B667-383921AD1D51}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="Z1" authorId="12" shapeId="0" xr:uid="{A8AB686C-C9A6-4D83-A065-3135BF12D8D4}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AA1" authorId="13" shapeId="0" xr:uid="{E58C168E-2BB7-4786-BE3F-79777D7D51A0}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AB1" authorId="14" shapeId="0" xr:uid="{73D3B685-456A-46FD-9453-FD680A256D7A}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AC1" authorId="15" shapeId="0" xr:uid="{79C7BAA5-FBAC-461E-A4C1-26EF533FE6C5}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AD1" authorId="16" shapeId="0" xr:uid="{213C33FB-B943-4920-A3B4-585B2F57EDE4}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AF1" authorId="17" shapeId="0" xr:uid="{B0634201-52B5-4EE6-9B76-BC0B1443B976}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AG1" authorId="18" shapeId="0" xr:uid="{237BA323-8F2B-4BED-B1DD-02DC08D0F310}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
@@ -245,153 +246,153 @@
   <commentList>
     <comment ref="F2" authorId="0" shapeId="0" xr:uid="{A0066626-C7AC-433A-812F-BA8F706B6CB3}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="G2" authorId="1" shapeId="0" xr:uid="{874FCA18-FCBE-4DDD-9292-A01B7619287C}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="H2" authorId="2" shapeId="0" xr:uid="{F6A9A9E8-413D-4EE0-B271-5836D62E0AFD}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="I2" authorId="3" shapeId="0" xr:uid="{E3DD0863-7811-45EE-AC49-4ED8766797CA}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="J2" authorId="4" shapeId="0" xr:uid="{7B31A9E4-E2F9-48FB-A088-3D7C7DB9B4E7}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     add per requested</t>
       </text>
     </comment>
     <comment ref="M2" authorId="5" shapeId="0" xr:uid="{3CD434D8-DB27-4523-B51A-09FCCA0B844E}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new add</t>
       </text>
     </comment>
     <comment ref="N2" authorId="6" shapeId="0" xr:uid="{BECDD6A5-3BEB-486E-97F5-93CF8BD76E9B}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new add</t>
       </text>
     </comment>
     <comment ref="P2" authorId="7" shapeId="0" xr:uid="{E6CCBEA7-FF92-4274-AC51-F78DA7A96792}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new add</t>
       </text>
     </comment>
     <comment ref="Q2" authorId="8" shapeId="0" xr:uid="{9F9AF825-C069-4839-B033-2A163E6C374A}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new add</t>
       </text>
     </comment>
     <comment ref="R2" authorId="9" shapeId="0" xr:uid="{E67154D2-87A9-467B-961B-AF2D4C5F8523}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="S2" authorId="10" shapeId="0" xr:uid="{6CEB863F-AD5D-424A-8C21-1AA4BE0F40B1}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="T2" authorId="11" shapeId="0" xr:uid="{A03B9F19-0397-4F91-B0B6-DB7392707278}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="Z2" authorId="12" shapeId="0" xr:uid="{DFBBA381-8A97-457F-BAF9-E6F6D4FF5103}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AA2" authorId="13" shapeId="0" xr:uid="{72A8297E-923A-4B99-A086-2610D7439DD9}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AB2" authorId="14" shapeId="0" xr:uid="{2DAC4C53-0F6F-4867-97F5-39055BD851BA}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AC2" authorId="15" shapeId="0" xr:uid="{9025DEF3-5CB6-44EC-B41D-B3E7F20E5527}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AD2" authorId="16" shapeId="0" xr:uid="{F4607535-4862-4883-93E8-0B66B130D3DA}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AF2" authorId="17" shapeId="0" xr:uid="{6D94C08D-35A5-49F7-ACC5-07AD678934AA}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
     <comment ref="AG2" authorId="18" shapeId="0" xr:uid="{B637D08A-B1EC-4ECD-A124-E8135720BADB}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
     new added</t>
       </text>
     </comment>
@@ -400,7 +401,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="140">
   <si>
     <t>Choice</t>
   </si>
@@ -768,57 +769,87 @@
     <t>PDS-DCP</t>
   </si>
   <si>
-    <t>XX公司</t>
-  </si>
-  <si>
-    <t>医院</t>
-  </si>
-  <si>
-    <t>医院商贸</t>
-  </si>
-  <si>
-    <t>不确定</t>
-  </si>
-  <si>
-    <t>33@philips.com</t>
-  </si>
-  <si>
-    <t>2022-4-01</t>
-  </si>
-  <si>
-    <t>2022-04-02</t>
-  </si>
-  <si>
-    <t>2022-4-18</t>
-  </si>
-  <si>
-    <t>2022-4-06</t>
-  </si>
-  <si>
-    <t>2022-04-09</t>
-  </si>
-  <si>
-    <t>2022-04/13</t>
-  </si>
-  <si>
-    <t>2022/4/06</t>
-  </si>
-  <si>
-    <t>2022/4-06</t>
-  </si>
-  <si>
-    <t>2022/04/09</t>
+    <t>可换货期订单销售</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>可换货期医院编号</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>产品线</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>订单Reference ID</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>订单类型</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>销售区域</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>业务模式</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>经销商编号</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>经销商</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>医院编号</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>医院名称</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>可换货期订单销售区域</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>可换货期医院名称</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>可换货期订单型号</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>可换货期订单SO#</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>可换货期订单WBS#</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>可换货期订单记认销售日期</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>xxx</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -826,7 +857,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -834,7 +865,7 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -842,17 +873,30 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -916,7 +960,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -972,11 +1016,12 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{DB8A74A6-6841-42AE-B314-497A4800DD25}"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="2" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -998,7 +1043,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1422,74 +1467,74 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AH16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9.125" style="1"/>
     <col min="2" max="3" width="23" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="23" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="19.28515625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.85546875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="21.28515625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" style="1"/>
-    <col min="14" max="14" width="13.28515625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="20.42578125" style="15" customWidth="1"/>
-    <col min="16" max="16" width="24.140625" style="15" customWidth="1"/>
+    <col min="7" max="7" width="16.875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.125" style="1"/>
+    <col min="14" max="14" width="13.375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="20.5" style="15" customWidth="1"/>
+    <col min="16" max="16" width="24.125" style="15" customWidth="1"/>
     <col min="17" max="17" width="19" style="15" customWidth="1"/>
-    <col min="18" max="18" width="21.5703125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="21.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="16.42578125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="11.7109375" style="15" customWidth="1"/>
-    <col min="22" max="22" width="12.5703125" style="15" customWidth="1"/>
-    <col min="23" max="23" width="13.42578125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="19.28515625" style="15" customWidth="1"/>
-    <col min="25" max="25" width="23.140625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="26.5703125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="18.28515625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="16.5703125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="21.7109375" style="1" customWidth="1"/>
-    <col min="30" max="30" width="27.140625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="24.5703125" style="1" customWidth="1"/>
-    <col min="32" max="32" width="27.140625" style="1" customWidth="1"/>
-    <col min="33" max="33" width="23.7109375" style="1" customWidth="1"/>
-    <col min="34" max="34" width="24.85546875" style="15" customWidth="1"/>
-    <col min="35" max="16384" width="9.140625" style="1"/>
+    <col min="18" max="18" width="21.5" style="1" customWidth="1"/>
+    <col min="19" max="19" width="21.125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="16.5" style="1" customWidth="1"/>
+    <col min="21" max="21" width="11.625" style="15" customWidth="1"/>
+    <col min="22" max="22" width="12.5" style="15" customWidth="1"/>
+    <col min="23" max="23" width="13.5" style="1" customWidth="1"/>
+    <col min="24" max="24" width="19.375" style="15" customWidth="1"/>
+    <col min="25" max="25" width="23.125" style="1" customWidth="1"/>
+    <col min="26" max="26" width="26.5" style="1" customWidth="1"/>
+    <col min="27" max="27" width="19.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21.625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="27.125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="24.5" style="1" customWidth="1"/>
+    <col min="32" max="32" width="27.125" style="1" customWidth="1"/>
+    <col min="33" max="33" width="23.625" style="1" customWidth="1"/>
+    <col min="34" max="34" width="24.875" style="15" customWidth="1"/>
+    <col min="35" max="16384" width="9.125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="38.25" customHeight="1">
+    <row r="1" spans="1:34" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>5</v>
+        <v>126</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>7</v>
+        <v>124</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>8</v>
+        <v>127</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>127</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>11</v>
+        <v>129</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>13</v>
+        <v>131</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>14</v>
+        <v>132</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>15</v>
@@ -1537,230 +1582,106 @@
         <v>27</v>
       </c>
       <c r="Z1" s="10" t="s">
-        <v>28</v>
+        <v>122</v>
       </c>
       <c r="AA1" s="10" t="s">
-        <v>29</v>
+        <v>133</v>
       </c>
       <c r="AB1" s="10" t="s">
-        <v>29</v>
+        <v>133</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>30</v>
+        <v>123</v>
       </c>
       <c r="AD1" s="10" t="s">
-        <v>31</v>
+        <v>134</v>
       </c>
       <c r="AE1" s="10" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="AF1" s="10" t="s">
-        <v>32</v>
+        <v>136</v>
       </c>
       <c r="AG1" s="10" t="s">
-        <v>33</v>
+        <v>137</v>
       </c>
       <c r="AH1" s="16" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="2" spans="1:34" ht="15">
-      <c r="A2" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1231231</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>48</v>
-      </c>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:34" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A2" s="5"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2" t="s">
-        <v>122</v>
-      </c>
+      <c r="H2" s="19"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="L2" s="2">
-        <v>1231</v>
-      </c>
-      <c r="M2" s="2">
-        <v>1231231</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="O2" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="P2" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q2" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="T2" s="2">
-        <v>1231231</v>
-      </c>
-      <c r="U2" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="V2" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="X2" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="Z2" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>47</v>
-      </c>
+      <c r="J2" s="19"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="8"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
-      <c r="AD2" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AF2" s="2">
-        <v>312312</v>
-      </c>
-      <c r="AG2" s="2">
-        <v>342342</v>
-      </c>
-      <c r="AH2" s="14" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="3" spans="1:34" ht="30">
-      <c r="A3" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="2">
-        <v>1231231</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="AD2" s="2"/>
+      <c r="AE2" s="2"/>
+      <c r="AF2" s="2"/>
+      <c r="AG2" s="2"/>
+      <c r="AH2" s="14"/>
+    </row>
+    <row r="3" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2" t="s">
-        <v>122</v>
-      </c>
+      <c r="H3" s="2"/>
       <c r="I3" s="2"/>
-      <c r="J3" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="L3" s="2">
-        <v>1231</v>
-      </c>
-      <c r="M3" s="2">
-        <v>1231231</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="O3" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="P3" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="Q3" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="R3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="T3" s="2">
-        <v>1231231</v>
-      </c>
-      <c r="U3" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="V3" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="X3" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="Z3" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="AA3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB3" s="2" t="s">
-        <v>47</v>
-      </c>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="14"/>
+      <c r="Q3" s="14"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="14"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="14"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="8"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
-      <c r="AD3" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE3" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="AF3" s="2">
-        <v>312312</v>
-      </c>
-      <c r="AG3" s="2">
-        <v>342341</v>
-      </c>
-      <c r="AH3" s="14" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="4" spans="1:34" ht="15">
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="14"/>
+    </row>
+    <row r="4" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="5"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1790,13 +1711,15 @@
       <c r="AA4" s="2"/>
       <c r="AB4" s="2"/>
       <c r="AC4" s="2"/>
-      <c r="AD4" s="2"/>
+      <c r="AD4" s="2" t="s">
+        <v>139</v>
+      </c>
       <c r="AE4" s="2"/>
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
       <c r="AH4" s="14"/>
     </row>
-    <row r="5" spans="1:34" ht="15">
+    <row r="5" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1832,7 +1755,7 @@
       <c r="AG5" s="2"/>
       <c r="AH5" s="14"/>
     </row>
-    <row r="6" spans="1:34" ht="15">
+    <row r="6" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1868,7 +1791,7 @@
       <c r="AG6" s="2"/>
       <c r="AH6" s="14"/>
     </row>
-    <row r="7" spans="1:34" ht="15">
+    <row r="7" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1904,7 +1827,7 @@
       <c r="AG7" s="2"/>
       <c r="AH7" s="14"/>
     </row>
-    <row r="8" spans="1:34" ht="15">
+    <row r="8" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1940,7 +1863,7 @@
       <c r="AG8" s="2"/>
       <c r="AH8" s="14"/>
     </row>
-    <row r="9" spans="1:34" ht="15">
+    <row r="9" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1976,7 +1899,7 @@
       <c r="AG9" s="2"/>
       <c r="AH9" s="14"/>
     </row>
-    <row r="10" spans="1:34" ht="15">
+    <row r="10" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2012,7 +1935,7 @@
       <c r="AG10" s="2"/>
       <c r="AH10" s="14"/>
     </row>
-    <row r="11" spans="1:34" ht="15">
+    <row r="11" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -2048,7 +1971,7 @@
       <c r="AG11" s="2"/>
       <c r="AH11" s="14"/>
     </row>
-    <row r="12" spans="1:34" ht="15">
+    <row r="12" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2084,7 +2007,7 @@
       <c r="AG12" s="2"/>
       <c r="AH12" s="14"/>
     </row>
-    <row r="13" spans="1:34" ht="15">
+    <row r="13" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -2120,7 +2043,7 @@
       <c r="AG13" s="2"/>
       <c r="AH13" s="14"/>
     </row>
-    <row r="14" spans="1:34" ht="15">
+    <row r="14" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2156,7 +2079,7 @@
       <c r="AG14" s="2"/>
       <c r="AH14" s="14"/>
     </row>
-    <row r="15" spans="1:34" ht="15">
+    <row r="15" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2192,7 +2115,7 @@
       <c r="AG15" s="2"/>
       <c r="AH15" s="14"/>
     </row>
-    <row r="16" spans="1:34" ht="15">
+    <row r="16" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2236,14 +2159,9 @@
       <formula1>INDIRECT(D4)</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="Z2" r:id="rId1" xr:uid="{4D702C1D-EE50-42F4-8E79-1407CB195B13}"/>
-    <hyperlink ref="Z3" r:id="rId2" xr:uid="{C9098AE3-7A77-4FEE-B8D3-045B68EA699E}"/>
-    <hyperlink ref="R3" r:id="rId3" xr:uid="{9E739D5A-1E57-4547-B408-9B23C9C5A2F6}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
-  <legacyDrawing r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="12">
@@ -2331,45 +2249,45 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AH19"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9.125" style="1"/>
     <col min="2" max="3" width="23" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="23" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="19.28515625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.85546875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="21.28515625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" style="1"/>
-    <col min="14" max="14" width="13.28515625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="20.42578125" style="15" customWidth="1"/>
-    <col min="16" max="16" width="24.140625" style="15" customWidth="1"/>
+    <col min="7" max="7" width="16.875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="19.375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.125" style="1"/>
+    <col min="14" max="14" width="13.375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="20.5" style="15" customWidth="1"/>
+    <col min="16" max="16" width="24.125" style="15" customWidth="1"/>
     <col min="17" max="17" width="19" style="15" customWidth="1"/>
-    <col min="18" max="18" width="21.5703125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="21.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="16.42578125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="11.7109375" style="15" customWidth="1"/>
-    <col min="22" max="22" width="12.5703125" style="15" customWidth="1"/>
-    <col min="23" max="23" width="13.42578125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="19.28515625" style="15" customWidth="1"/>
-    <col min="25" max="25" width="23.140625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="26.5703125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="18.28515625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="16.5703125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="21.7109375" style="1" customWidth="1"/>
-    <col min="30" max="30" width="27.140625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="24.5703125" style="1" customWidth="1"/>
-    <col min="32" max="32" width="27.140625" style="1" customWidth="1"/>
-    <col min="33" max="33" width="23.7109375" style="1" customWidth="1"/>
-    <col min="34" max="34" width="24.85546875" style="15" customWidth="1"/>
-    <col min="35" max="16384" width="9.140625" style="1"/>
+    <col min="18" max="18" width="21.5" style="1" customWidth="1"/>
+    <col min="19" max="19" width="21.125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="16.5" style="1" customWidth="1"/>
+    <col min="21" max="21" width="11.625" style="15" customWidth="1"/>
+    <col min="22" max="22" width="12.5" style="15" customWidth="1"/>
+    <col min="23" max="23" width="13.5" style="1" customWidth="1"/>
+    <col min="24" max="24" width="19.375" style="15" customWidth="1"/>
+    <col min="25" max="25" width="23.125" style="1" customWidth="1"/>
+    <col min="26" max="26" width="26.5" style="1" customWidth="1"/>
+    <col min="27" max="27" width="18.375" style="1" customWidth="1"/>
+    <col min="28" max="28" width="16.5" style="1" customWidth="1"/>
+    <col min="29" max="29" width="21.625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="27.125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="24.5" style="1" customWidth="1"/>
+    <col min="32" max="32" width="27.125" style="1" customWidth="1"/>
+    <col min="33" max="33" width="23.625" style="1" customWidth="1"/>
+    <col min="34" max="34" width="24.875" style="15" customWidth="1"/>
+    <col min="35" max="16384" width="9.125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="17.25" customHeight="1">
+    <row r="1" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2470,7 +2388,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="38.25" customHeight="1">
+    <row r="2" spans="1:34" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>5</v>
       </c>
@@ -2574,7 +2492,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="15">
+    <row r="3" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>34</v>
       </c>
@@ -2636,7 +2554,7 @@
       <c r="AG3" s="2"/>
       <c r="AH3" s="14"/>
     </row>
-    <row r="4" spans="1:34">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A4" s="5"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -2672,7 +2590,7 @@
       <c r="AG4" s="2"/>
       <c r="AH4" s="14"/>
     </row>
-    <row r="5" spans="1:34">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -2708,7 +2626,7 @@
       <c r="AG5" s="5"/>
       <c r="AH5" s="18"/>
     </row>
-    <row r="6" spans="1:34">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -2744,7 +2662,7 @@
       <c r="AG6" s="5"/>
       <c r="AH6" s="18"/>
     </row>
-    <row r="7" spans="1:34">
+    <row r="7" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -2780,7 +2698,7 @@
       <c r="AG7" s="5"/>
       <c r="AH7" s="18"/>
     </row>
-    <row r="8" spans="1:34">
+    <row r="8" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -2816,7 +2734,7 @@
       <c r="AG8" s="5"/>
       <c r="AH8" s="18"/>
     </row>
-    <row r="9" spans="1:34">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -2852,7 +2770,7 @@
       <c r="AG9" s="5"/>
       <c r="AH9" s="18"/>
     </row>
-    <row r="10" spans="1:34">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -2888,7 +2806,7 @@
       <c r="AG10" s="5"/>
       <c r="AH10" s="18"/>
     </row>
-    <row r="11" spans="1:34">
+    <row r="11" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -2924,7 +2842,7 @@
       <c r="AG11" s="5"/>
       <c r="AH11" s="18"/>
     </row>
-    <row r="12" spans="1:34">
+    <row r="12" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -2960,7 +2878,7 @@
       <c r="AG12" s="5"/>
       <c r="AH12" s="18"/>
     </row>
-    <row r="13" spans="1:34">
+    <row r="13" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -2996,7 +2914,7 @@
       <c r="AG13" s="5"/>
       <c r="AH13" s="18"/>
     </row>
-    <row r="14" spans="1:34">
+    <row r="14" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -3032,7 +2950,7 @@
       <c r="AG14" s="5"/>
       <c r="AH14" s="18"/>
     </row>
-    <row r="15" spans="1:34">
+    <row r="15" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -3068,7 +2986,7 @@
       <c r="AG15" s="5"/>
       <c r="AH15" s="18"/>
     </row>
-    <row r="16" spans="1:34">
+    <row r="16" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -3104,7 +3022,7 @@
       <c r="AG16" s="5"/>
       <c r="AH16" s="18"/>
     </row>
-    <row r="17" spans="1:34">
+    <row r="17" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -3140,11 +3058,12 @@
       <c r="AG17" s="5"/>
       <c r="AH17" s="18"/>
     </row>
-    <row r="19" spans="1:34">
+    <row r="19" spans="1:34" x14ac:dyDescent="0.2">
       <c r="T19" s="12"/>
     </row>
   </sheetData>
   <autoFilter ref="B2:AP2" xr:uid="{47CA263F-3211-4E45-A5EC-F4F3FE6D73B4}"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="Z3" r:id="rId1" xr:uid="{7835CF24-7111-425A-BBC9-C6FF2381CDB3}"/>
   </hyperlinks>
@@ -3235,15 +3154,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60B8DC03-3E4A-4D59-A3C8-4981847DA953}">
   <dimension ref="A1:O28"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="3" width="15.5703125" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="2" max="3" width="15.5" customWidth="1"/>
+    <col min="4" max="4" width="12.375" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>34</v>
       </c>
@@ -3284,7 +3203,7 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>53</v>
       </c>
@@ -3323,7 +3242,7 @@
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>60</v>
@@ -3354,7 +3273,7 @@
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>62</v>
@@ -3385,7 +3304,7 @@
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>65</v>
@@ -3416,7 +3335,7 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -3447,7 +3366,7 @@
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>75</v>
@@ -3476,7 +3395,7 @@
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
         <v>79</v>
@@ -3505,7 +3424,7 @@
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>83</v>
       </c>
@@ -3522,7 +3441,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>121</v>
       </c>
@@ -3539,7 +3458,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>35</v>
       </c>
@@ -3556,7 +3475,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>87</v>
       </c>
@@ -3573,7 +3492,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>92</v>
       </c>
@@ -3590,7 +3509,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>95</v>
       </c>
@@ -3607,7 +3526,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>98</v>
       </c>
@@ -3624,7 +3543,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>101</v>
       </c>
@@ -3638,7 +3557,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="4:10">
+    <row r="17" spans="4:10" x14ac:dyDescent="0.2">
       <c r="D17" t="s">
         <v>87</v>
       </c>
@@ -3646,7 +3565,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="4:10">
+    <row r="18" spans="4:10" x14ac:dyDescent="0.2">
       <c r="D18" t="s">
         <v>92</v>
       </c>
@@ -3654,7 +3573,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="4:10">
+    <row r="19" spans="4:10" x14ac:dyDescent="0.2">
       <c r="D19" t="s">
         <v>95</v>
       </c>
@@ -3662,7 +3581,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="4:10">
+    <row r="20" spans="4:10" x14ac:dyDescent="0.2">
       <c r="D20" t="s">
         <v>98</v>
       </c>
@@ -3670,7 +3589,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="4:10">
+    <row r="21" spans="4:10" x14ac:dyDescent="0.2">
       <c r="D21" t="s">
         <v>101</v>
       </c>
@@ -3678,59 +3597,60 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="4:10">
+    <row r="22" spans="4:10" x14ac:dyDescent="0.2">
       <c r="J22" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="23" spans="4:10">
+    <row r="23" spans="4:10" x14ac:dyDescent="0.2">
       <c r="J23" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="24" spans="4:10">
+    <row r="24" spans="4:10" x14ac:dyDescent="0.2">
       <c r="J24" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="25" spans="4:10">
+    <row r="25" spans="4:10" x14ac:dyDescent="0.2">
       <c r="J25" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="26" spans="4:10">
+    <row r="26" spans="4:10" x14ac:dyDescent="0.2">
       <c r="J26" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="27" spans="4:10">
+    <row r="27" spans="4:10" x14ac:dyDescent="0.2">
       <c r="J27" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="28" spans="4:10">
+    <row r="28" spans="4:10" x14ac:dyDescent="0.2">
       <c r="J28" t="s">
         <v>116</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3925,18 +3845,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{170FD28C-CD37-430A-A401-4A184398A888}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0415A386-986E-4768-9558-FCE8C9749E25}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0415A386-986E-4768-9558-FCE8C9749E25}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{170FD28C-CD37-430A-A401-4A184398A888}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
fix: [special approval] rdd_oit field limit
</commit_message>
<xml_diff>
--- a/src/assets/template/RDD-OIT-180-Template.xlsx
+++ b/src/assets/template/RDD-OIT-180-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1C7867-598C-463B-AA01-AC07CD155279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564389C5-F722-4A18-98A0-7E5719F440BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{A3335066-89F2-47A1-BD65-2F9EA0750B57}"/>
   </bookViews>
@@ -22,7 +22,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RDD&gt; 180 with fields Type'!$B$2:$AP$2</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -401,7 +400,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="139">
   <si>
     <t>Choice</t>
   </si>
@@ -834,10 +833,6 @@
   </si>
   <si>
     <t>可换货期订单记认销售日期</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>xxx</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -1467,45 +1462,45 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AH16"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.125" style="1"/>
+    <col min="1" max="1" width="9.109375" style="1"/>
     <col min="2" max="3" width="23" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="23" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="22.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="21.375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9.125" style="1"/>
-    <col min="14" max="14" width="13.375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="20.5" style="15" customWidth="1"/>
-    <col min="16" max="16" width="24.125" style="15" customWidth="1"/>
+    <col min="7" max="7" width="16.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.33203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.109375" style="1"/>
+    <col min="14" max="14" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="20.44140625" style="15" customWidth="1"/>
+    <col min="16" max="16" width="24.109375" style="15" customWidth="1"/>
     <col min="17" max="17" width="19" style="15" customWidth="1"/>
-    <col min="18" max="18" width="21.5" style="1" customWidth="1"/>
-    <col min="19" max="19" width="21.125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="16.5" style="1" customWidth="1"/>
-    <col min="21" max="21" width="11.625" style="15" customWidth="1"/>
-    <col min="22" max="22" width="12.5" style="15" customWidth="1"/>
-    <col min="23" max="23" width="13.5" style="1" customWidth="1"/>
-    <col min="24" max="24" width="19.375" style="15" customWidth="1"/>
-    <col min="25" max="25" width="23.125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="26.5" style="1" customWidth="1"/>
-    <col min="27" max="27" width="19.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="21.625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="27.125" style="1" customWidth="1"/>
-    <col min="31" max="31" width="24.5" style="1" customWidth="1"/>
-    <col min="32" max="32" width="27.125" style="1" customWidth="1"/>
-    <col min="33" max="33" width="23.625" style="1" customWidth="1"/>
-    <col min="34" max="34" width="24.875" style="15" customWidth="1"/>
-    <col min="35" max="16384" width="9.125" style="1"/>
+    <col min="18" max="18" width="21.44140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="21.109375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="16.44140625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="11.6640625" style="15" customWidth="1"/>
+    <col min="22" max="22" width="12.44140625" style="15" customWidth="1"/>
+    <col min="23" max="23" width="13.44140625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="19.33203125" style="15" customWidth="1"/>
+    <col min="25" max="25" width="23.109375" style="1" customWidth="1"/>
+    <col min="26" max="26" width="26.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21.6640625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="27.109375" style="1" customWidth="1"/>
+    <col min="31" max="31" width="24.44140625" style="1" customWidth="1"/>
+    <col min="32" max="32" width="27.109375" style="1" customWidth="1"/>
+    <col min="33" max="33" width="23.6640625" style="1" customWidth="1"/>
+    <col min="34" max="34" width="24.88671875" style="15" customWidth="1"/>
+    <col min="35" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:34" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>126</v>
       </c>
@@ -1609,7 +1604,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1645,7 +1640,7 @@
       <c r="AG2" s="2"/>
       <c r="AH2" s="14"/>
     </row>
-    <row r="3" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1681,7 +1676,7 @@
       <c r="AG3" s="2"/>
       <c r="AH3" s="14"/>
     </row>
-    <row r="4" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1711,15 +1706,13 @@
       <c r="AA4" s="2"/>
       <c r="AB4" s="2"/>
       <c r="AC4" s="2"/>
-      <c r="AD4" s="2" t="s">
-        <v>139</v>
-      </c>
+      <c r="AD4" s="2"/>
       <c r="AE4" s="2"/>
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
       <c r="AH4" s="14"/>
     </row>
-    <row r="5" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1755,7 +1748,7 @@
       <c r="AG5" s="2"/>
       <c r="AH5" s="14"/>
     </row>
-    <row r="6" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1791,7 +1784,7 @@
       <c r="AG6" s="2"/>
       <c r="AH6" s="14"/>
     </row>
-    <row r="7" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1827,7 +1820,7 @@
       <c r="AG7" s="2"/>
       <c r="AH7" s="14"/>
     </row>
-    <row r="8" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1863,7 +1856,7 @@
       <c r="AG8" s="2"/>
       <c r="AH8" s="14"/>
     </row>
-    <row r="9" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1899,7 +1892,7 @@
       <c r="AG9" s="2"/>
       <c r="AH9" s="14"/>
     </row>
-    <row r="10" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1935,7 +1928,7 @@
       <c r="AG10" s="2"/>
       <c r="AH10" s="14"/>
     </row>
-    <row r="11" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1971,7 +1964,7 @@
       <c r="AG11" s="2"/>
       <c r="AH11" s="14"/>
     </row>
-    <row r="12" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2007,7 +2000,7 @@
       <c r="AG12" s="2"/>
       <c r="AH12" s="14"/>
     </row>
-    <row r="13" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -2043,7 +2036,7 @@
       <c r="AG13" s="2"/>
       <c r="AH13" s="14"/>
     </row>
-    <row r="14" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2079,7 +2072,7 @@
       <c r="AG14" s="2"/>
       <c r="AH14" s="14"/>
     </row>
-    <row r="15" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2115,7 +2108,7 @@
       <c r="AG15" s="2"/>
       <c r="AH15" s="14"/>
     </row>
-    <row r="16" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2249,45 +2242,45 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AH19"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.125" style="1"/>
+    <col min="1" max="1" width="9.109375" style="1"/>
     <col min="2" max="3" width="23" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="23" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5" style="1" customWidth="1"/>
-    <col min="9" max="9" width="19.375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="21.375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9.125" style="1"/>
-    <col min="14" max="14" width="13.375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="20.5" style="15" customWidth="1"/>
-    <col min="16" max="16" width="24.125" style="15" customWidth="1"/>
+    <col min="7" max="7" width="16.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.44140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.33203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.109375" style="1"/>
+    <col min="14" max="14" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="20.44140625" style="15" customWidth="1"/>
+    <col min="16" max="16" width="24.109375" style="15" customWidth="1"/>
     <col min="17" max="17" width="19" style="15" customWidth="1"/>
-    <col min="18" max="18" width="21.5" style="1" customWidth="1"/>
-    <col min="19" max="19" width="21.125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="16.5" style="1" customWidth="1"/>
-    <col min="21" max="21" width="11.625" style="15" customWidth="1"/>
-    <col min="22" max="22" width="12.5" style="15" customWidth="1"/>
-    <col min="23" max="23" width="13.5" style="1" customWidth="1"/>
-    <col min="24" max="24" width="19.375" style="15" customWidth="1"/>
-    <col min="25" max="25" width="23.125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="26.5" style="1" customWidth="1"/>
-    <col min="27" max="27" width="18.375" style="1" customWidth="1"/>
-    <col min="28" max="28" width="16.5" style="1" customWidth="1"/>
-    <col min="29" max="29" width="21.625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="27.125" style="1" customWidth="1"/>
-    <col min="31" max="31" width="24.5" style="1" customWidth="1"/>
-    <col min="32" max="32" width="27.125" style="1" customWidth="1"/>
-    <col min="33" max="33" width="23.625" style="1" customWidth="1"/>
-    <col min="34" max="34" width="24.875" style="15" customWidth="1"/>
-    <col min="35" max="16384" width="9.125" style="1"/>
+    <col min="18" max="18" width="21.44140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="21.109375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="16.44140625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="11.6640625" style="15" customWidth="1"/>
+    <col min="22" max="22" width="12.44140625" style="15" customWidth="1"/>
+    <col min="23" max="23" width="13.44140625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="19.33203125" style="15" customWidth="1"/>
+    <col min="25" max="25" width="23.109375" style="1" customWidth="1"/>
+    <col min="26" max="26" width="26.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="18.33203125" style="1" customWidth="1"/>
+    <col min="28" max="28" width="16.44140625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="21.6640625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="27.109375" style="1" customWidth="1"/>
+    <col min="31" max="31" width="24.44140625" style="1" customWidth="1"/>
+    <col min="32" max="32" width="27.109375" style="1" customWidth="1"/>
+    <col min="33" max="33" width="23.6640625" style="1" customWidth="1"/>
+    <col min="34" max="34" width="24.88671875" style="15" customWidth="1"/>
+    <col min="35" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2388,7 +2381,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:34" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>5</v>
       </c>
@@ -2492,7 +2485,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>34</v>
       </c>
@@ -2554,7 +2547,7 @@
       <c r="AG3" s="2"/>
       <c r="AH3" s="14"/>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -2590,7 +2583,7 @@
       <c r="AG4" s="2"/>
       <c r="AH4" s="14"/>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -2626,7 +2619,7 @@
       <c r="AG5" s="5"/>
       <c r="AH5" s="18"/>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -2662,7 +2655,7 @@
       <c r="AG6" s="5"/>
       <c r="AH6" s="18"/>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -2698,7 +2691,7 @@
       <c r="AG7" s="5"/>
       <c r="AH7" s="18"/>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -2734,7 +2727,7 @@
       <c r="AG8" s="5"/>
       <c r="AH8" s="18"/>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -2770,7 +2763,7 @@
       <c r="AG9" s="5"/>
       <c r="AH9" s="18"/>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -2806,7 +2799,7 @@
       <c r="AG10" s="5"/>
       <c r="AH10" s="18"/>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -2842,7 +2835,7 @@
       <c r="AG11" s="5"/>
       <c r="AH11" s="18"/>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -2878,7 +2871,7 @@
       <c r="AG12" s="5"/>
       <c r="AH12" s="18"/>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -2914,7 +2907,7 @@
       <c r="AG13" s="5"/>
       <c r="AH13" s="18"/>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -2950,7 +2943,7 @@
       <c r="AG14" s="5"/>
       <c r="AH14" s="18"/>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -2986,7 +2979,7 @@
       <c r="AG15" s="5"/>
       <c r="AH15" s="18"/>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -3022,7 +3015,7 @@
       <c r="AG16" s="5"/>
       <c r="AH16" s="18"/>
     </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -3058,7 +3051,7 @@
       <c r="AG17" s="5"/>
       <c r="AH17" s="18"/>
     </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
       <c r="T19" s="12"/>
     </row>
   </sheetData>
@@ -3154,15 +3147,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60B8DC03-3E4A-4D59-A3C8-4981847DA953}">
   <dimension ref="A1:O28"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="15.5" customWidth="1"/>
-    <col min="4" max="4" width="12.375" customWidth="1"/>
+    <col min="2" max="3" width="15.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="10" max="10" width="13.375" customWidth="1"/>
+    <col min="10" max="10" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>34</v>
       </c>
@@ -3203,7 +3196,7 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>53</v>
       </c>
@@ -3242,7 +3235,7 @@
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>60</v>
@@ -3273,7 +3266,7 @@
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>62</v>
@@ -3304,7 +3297,7 @@
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>65</v>
@@ -3335,7 +3328,7 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>70</v>
@@ -3366,7 +3359,7 @@
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>75</v>
@@ -3395,7 +3388,7 @@
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
         <v>79</v>
@@ -3424,7 +3417,7 @@
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>83</v>
       </c>
@@ -3441,7 +3434,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>121</v>
       </c>
@@ -3458,7 +3451,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>35</v>
       </c>
@@ -3475,7 +3468,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>87</v>
       </c>
@@ -3492,7 +3485,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>92</v>
       </c>
@@ -3509,7 +3502,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>95</v>
       </c>
@@ -3526,7 +3519,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>98</v>
       </c>
@@ -3543,7 +3536,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>101</v>
       </c>
@@ -3557,7 +3550,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
         <v>87</v>
       </c>
@@ -3565,7 +3558,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
         <v>92</v>
       </c>
@@ -3573,7 +3566,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
         <v>95</v>
       </c>
@@ -3581,7 +3574,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
         <v>98</v>
       </c>
@@ -3589,7 +3582,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
         <v>101</v>
       </c>
@@ -3597,37 +3590,37 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J22" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="23" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J23" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="24" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J24" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="25" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="26" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="27" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="28" spans="4:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
         <v>116</v>
       </c>
@@ -3639,18 +3632,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3845,18 +3838,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0415A386-986E-4768-9558-FCE8C9749E25}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{170FD28C-CD37-430A-A401-4A184398A888}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{170FD28C-CD37-430A-A401-4A184398A888}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0415A386-986E-4768-9558-FCE8C9749E25}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
fix: [special approval] #3103, #3155, #3156
</commit_message>
<xml_diff>
--- a/src/assets/template/RDD-OIT-180-Template.xlsx
+++ b/src/assets/template/RDD-OIT-180-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564389C5-F722-4A18-98A0-7E5719F440BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D5828D-B9B1-4B2D-A79E-FA2ECC3F5033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{A3335066-89F2-47A1-BD65-2F9EA0750B57}"/>
   </bookViews>
@@ -561,9 +561,6 @@
     <t>anna.zhu@philips.com</t>
   </si>
   <si>
-    <t>Pre-Book</t>
-  </si>
-  <si>
     <t>CT</t>
   </si>
   <si>
@@ -834,6 +831,10 @@
   <si>
     <t>可换货期订单记认销售日期</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pre-book</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1502,34 +1503,34 @@
   <sheetData>
     <row r="1" spans="1:34" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>132</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>15</v>
@@ -1559,10 +1560,10 @@
         <v>23</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="U1" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="V1" s="13" t="s">
         <v>24</v>
@@ -1577,31 +1578,31 @@
         <v>27</v>
       </c>
       <c r="Z1" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="AA1" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="AB1" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="AC1" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="AA1" s="10" t="s">
+      <c r="AD1" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="AB1" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="AD1" s="10" t="s">
+      <c r="AE1" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="AE1" s="10" t="s">
+      <c r="AF1" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="AF1" s="10" t="s">
+      <c r="AG1" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="AG1" s="10" t="s">
+      <c r="AH1" s="16" t="s">
         <v>137</v>
-      </c>
-      <c r="AH1" s="16" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
@@ -2147,34 +2148,17 @@
   </sheetData>
   <autoFilter ref="B1:AP1" xr:uid="{47CA263F-3211-4E45-A5EC-F4F3FE6D73B4}"/>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E16" xr:uid="{962478D9-B82A-4FB5-84D6-ADC33EFE10D2}">
-      <formula1>INDIRECT(D4)</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="12">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D2CA9823-178A-4080-91E0-4BE44777A068}">
-          <x14:formula1>
-            <xm:f>DropdownList!$D:$D</xm:f>
-          </x14:formula1>
-          <xm:sqref>AA2:AA16</xm:sqref>
-        </x14:dataValidation>
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="10">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7139D1AF-4E71-450F-ADAF-881C9742367D}">
           <x14:formula1>
             <xm:f>DropdownList!$J:$J</xm:f>
           </x14:formula1>
           <xm:sqref>S2:S16</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B5F05591-E095-4C19-BB54-18296E17428D}">
-          <x14:formula1>
-            <xm:f>DropdownList!$E:$E</xm:f>
-          </x14:formula1>
-          <xm:sqref>AB2:AB16</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1C833165-6109-41A5-A158-159AEE943A61}">
           <x14:formula1>
@@ -2186,7 +2170,7 @@
           <x14:formula1>
             <xm:f>DropdownList!$D$1:$D$21</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D16</xm:sqref>
+          <xm:sqref>D2:D1048576 AA2:AA1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9633456E-42A7-4FB8-8842-C55D2CE57DA6}">
           <x14:formula1>
@@ -2222,7 +2206,7 @@
           <x14:formula1>
             <xm:f>DropdownList!$E$1:$E$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E3</xm:sqref>
+          <xm:sqref>E2:E1048576 AB2:AB1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9CD28F98-72BF-4C21-955A-F56804185F25}">
           <x14:formula1>
@@ -2440,10 +2424,10 @@
         <v>23</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="U2" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="V2" s="13" t="s">
         <v>24</v>
@@ -2473,7 +2457,7 @@
         <v>31</v>
       </c>
       <c r="AE2" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AF2" s="10" t="s">
         <v>32</v>
@@ -2482,7 +2466,7 @@
         <v>33</v>
       </c>
       <c r="AH2" s="16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
@@ -2497,7 +2481,7 @@
         <v>35</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>37</v>
@@ -2510,7 +2494,7 @@
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O3" s="14"/>
       <c r="P3" s="14"/>
@@ -3198,38 +3182,38 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>37</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="K2" s="7" t="s">
         <v>40</v>
       </c>
       <c r="L2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
@@ -3238,7 +3222,7 @@
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>46</v>
@@ -3251,7 +3235,7 @@
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -3260,7 +3244,7 @@
       </c>
       <c r="K3" s="1"/>
       <c r="L3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
@@ -3269,16 +3253,16 @@
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
@@ -3287,7 +3271,7 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" t="s">
@@ -3300,16 +3284,16 @@
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5" t="s">
         <v>66</v>
-      </c>
-      <c r="E5" t="s">
-        <v>67</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
@@ -3318,11 +3302,11 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
@@ -3331,20 +3315,20 @@
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" t="s">
         <v>71</v>
-      </c>
-      <c r="E6" t="s">
-        <v>72</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -3353,7 +3337,7 @@
       </c>
       <c r="K6" s="1"/>
       <c r="L6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
@@ -3362,27 +3346,27 @@
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
@@ -3391,27 +3375,27 @@
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
@@ -3419,36 +3403,36 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E9" t="s">
         <v>36</v>
       </c>
       <c r="J9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -3456,197 +3440,183 @@
         <v>35</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" t="s">
         <v>88</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>89</v>
       </c>
-      <c r="E11" t="s">
+      <c r="J11" t="s">
         <v>90</v>
-      </c>
-      <c r="J11" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>88</v>
       </c>
       <c r="D12" t="s">
         <v>43</v>
       </c>
       <c r="E12" t="s">
+        <v>92</v>
+      </c>
+      <c r="J12" t="s">
         <v>93</v>
-      </c>
-      <c r="J12" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
+        <v>95</v>
+      </c>
+      <c r="J13" t="s">
         <v>96</v>
-      </c>
-      <c r="J13" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D14" t="s">
+        <v>98</v>
+      </c>
+      <c r="E14" t="s">
+        <v>94</v>
+      </c>
+      <c r="J14" t="s">
         <v>99</v>
-      </c>
-      <c r="E14" t="s">
-        <v>95</v>
-      </c>
-      <c r="J14" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D15" t="s">
+        <v>101</v>
+      </c>
+      <c r="E15" t="s">
+        <v>97</v>
+      </c>
+      <c r="J15" t="s">
         <v>102</v>
-      </c>
-      <c r="E15" t="s">
-        <v>98</v>
-      </c>
-      <c r="J15" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D16" t="s">
         <v>35</v>
       </c>
       <c r="E16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J20" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J24" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" spans="4:10" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E13816111B82DE40ADDAD0D50DEE851D" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="98c5d7584c7fdc80e391c7606f30523b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4f3cd097-2d9a-46cb-8444-c2cb22decb26" xmlns:ns3="49432d69-91bf-4956-a0e7-dbf2ba0ff8c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4c9766d4a4f8e78a4086627875829706" ns2:_="" ns3:_="">
     <xsd:import namespace="4f3cd097-2d9a-46cb-8444-c2cb22decb26"/>
@@ -3837,24 +3807,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{170FD28C-CD37-430A-A401-4A184398A888}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0415A386-986E-4768-9558-FCE8C9749E25}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DC742CE-A2A2-46AA-9E33-C408ACAD85BC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3871,4 +3839,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{170FD28C-CD37-430A-A401-4A184398A888}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0415A386-986E-4768-9558-FCE8C9749E25}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>